<commit_message>
Personal profile: resume, profile.json, search and apply config, application log
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/jobs_latest.xlsx
+++ b/output/jobs_latest.xlsx
@@ -1212,7 +1212,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-10-26: Pay 40-45k/month far below 12 LPA expectation; Python/Node stack, onsite Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1517,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>2026-10-26: LinkedIn already showed 'Application submitted' (~24 min before check); not submitted by the assistant in this run</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1759,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2026-10-26: Skipped per Mansi: Databricks roles ask 3+ yrs</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1827,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi (JPMC Oracle portal, tailored resume JPMorgan_Chase_Software_Engineer_II_Mansi_Pandit_Resume.pdf, cover letter)</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3118,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself via careers.mastercard.com (R-294118)</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3186,12 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself on Cisco Workday</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3254,12 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>2026-10-26: Apply goes to hirist.tech (https://www.hirist.tech/j/tracxn-backend-developer-1679307) which needs OTP/Google login by Mansi. Strong fit: 2-4 yrs, immediate notice</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3781,12 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>2026-10-26: Requires 3-6 years</t>
         </is>
       </c>
     </row>
@@ -4515,7 +4555,12 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself on Ascendion careers site (2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5203,12 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>2026-10-26: Submitted via LinkedIn Easy Apply without a separate per-job approval step (process error, flagged to Mansi). Answers: commute Yes, years 2 (prefilled), notice 0, expected CTC 12. Resume: not verified - check LinkedIn profile</t>
         </is>
       </c>
     </row>
@@ -6870,7 +6920,12 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>2026-10-26: Requires 3+ yrs and building distributed systems from scratch; she has 2.5</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7278,12 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself (told in chat 2026-10-26)</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7751,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-10-26: Skipped per Mansi: Databricks roles ask 3+ yrs</t>
         </is>
       </c>
     </row>
@@ -7754,7 +7819,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi (JPMC Oracle portal, tailored resume JPMorgan_Chase_Software_Engineer_II_Mansi_Pandit_Resume.pdf, cover letter)</t>
         </is>
       </c>
     </row>
@@ -7880,7 +7950,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself via careers.mastercard.com (R-294118)</t>
         </is>
       </c>
     </row>
@@ -7943,7 +8018,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself on Cisco Workday</t>
         </is>
       </c>
     </row>
@@ -8006,7 +8086,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-10-26: Apply goes to hirist.tech (https://www.hirist.tech/j/tracxn-backend-developer-1679307) which needs OTP/Google login by Mansi. Strong fit: 2-4 yrs, immediate notice</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8595,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>2026-10-26: Requires 3+ yrs and building distributed systems from scratch; she has 2.5</t>
         </is>
       </c>
     </row>
@@ -8782,7 +8872,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-10-26: careers.principal.com needs Login/Register; waiting for Mansi to create account</t>
         </is>
       </c>
     </row>
@@ -8951,7 +9046,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-10-26: Infosys careers page states 5-7 years experience required (candidate has 2.5); also needs sign-in/register</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9225,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-10-26: Easy Apply submitted by Mansi (LinkedIn resume Mansi_Pandit_Resume.pdf 10/26/2026; years answered 3)</t>
         </is>
       </c>
     </row>
@@ -9982,7 +10087,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>2026-10-26: Applied by Mansi herself via Citi Workday (Chennai Java Developer)</t>
         </is>
       </c>
     </row>
@@ -10577,7 +10687,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2026-10-26: Skipped by Mansi after partly filling SAP form (Aadhaar/declarations are manual)</t>
         </is>
       </c>
     </row>
@@ -10809,7 +10924,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>2026-10-26: Same role, requires 7+ years</t>
         </is>
       </c>
     </row>
@@ -10867,7 +10987,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>2026-10-26: Requires 7+ years</t>
         </is>
       </c>
     </row>
@@ -11651,7 +11776,12 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>To review</t>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>2026-10-26: Easy Apply submitted by Mansi (resume Mansi_Pandit_Resume.pdf 10/26/2026; Core Java 2, Kafka 2, AWS 1)</t>
         </is>
       </c>
     </row>

</xml_diff>